<commit_message>
WIP: Gain_buff 节点 + 场景/预制体/Spine 本地改动
</commit_message>
<xml_diff>
--- a/DataTables/Datas/animationstate.xlsx
+++ b/DataTables/Datas/animationstate.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1">
@@ -907,18 +907,18 @@
     </row>
     <row r="25">
       <c r="B25" t="n">
-        <v>3000</v>
+        <v>2003</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>idle1</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -926,18 +926,18 @@
     </row>
     <row r="26">
       <c r="B26" t="n">
-        <v>3001</v>
+        <v>2004</v>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>idle2</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -945,18 +945,18 @@
     </row>
     <row r="27">
       <c r="B27" t="n">
-        <v>3002</v>
+        <v>2005</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>throw</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -964,18 +964,18 @@
     </row>
     <row r="28">
       <c r="B28" t="n">
-        <v>4000</v>
+        <v>2006</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>die</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -983,14 +983,14 @@
     </row>
     <row r="29">
       <c r="B29" t="n">
-        <v>4001</v>
+        <v>3001</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>talk</t>
+          <t>idle2</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1002,14 +1002,14 @@
     </row>
     <row r="30">
       <c r="B30" t="n">
-        <v>4002</v>
+        <v>3008</v>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>talk2</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1021,14 +1021,14 @@
     </row>
     <row r="31">
       <c r="B31" t="n">
-        <v>5000</v>
+        <v>3009</v>
       </c>
       <c r="C31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1040,14 +1040,14 @@
     </row>
     <row r="32">
       <c r="B32" t="n">
-        <v>5001</v>
+        <v>3010</v>
       </c>
       <c r="C32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>think1</t>
+          <t>attack2</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1059,14 +1059,14 @@
     </row>
     <row r="33">
       <c r="B33" t="n">
-        <v>5002</v>
+        <v>3011</v>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>talk</t>
+          <t>attack3</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1078,14 +1078,14 @@
     </row>
     <row r="34">
       <c r="B34" t="n">
-        <v>5003</v>
+        <v>3012</v>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>idle1</t>
+          <t>dead</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1097,14 +1097,14 @@
     </row>
     <row r="35">
       <c r="B35" t="n">
-        <v>6000</v>
+        <v>3013</v>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>die</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1116,14 +1116,14 @@
     </row>
     <row r="36">
       <c r="B36" t="n">
-        <v>6001</v>
+        <v>3014</v>
       </c>
       <c r="C36" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>think1</t>
+          <t>hurt</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1135,14 +1135,14 @@
     </row>
     <row r="37">
       <c r="B37" t="n">
-        <v>6002</v>
+        <v>3015</v>
       </c>
       <c r="C37" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>talk</t>
+          <t>hurt1</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1154,14 +1154,14 @@
     </row>
     <row r="38">
       <c r="B38" t="n">
-        <v>6003</v>
+        <v>3016</v>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>talk2</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1173,18 +1173,18 @@
     </row>
     <row r="39">
       <c r="B39" t="n">
-        <v>6004</v>
+        <v>3003</v>
       </c>
       <c r="C39" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>idle1</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1192,18 +1192,18 @@
     </row>
     <row r="40">
       <c r="B40" t="n">
-        <v>7000</v>
+        <v>3004</v>
       </c>
       <c r="C40" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -1211,10 +1211,10 @@
     </row>
     <row r="41">
       <c r="B41" t="n">
-        <v>7001</v>
+        <v>3005</v>
       </c>
       <c r="C41" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1230,18 +1230,18 @@
     </row>
     <row r="42">
       <c r="B42" t="n">
-        <v>7002</v>
+        <v>3006</v>
       </c>
       <c r="C42" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>attack2</t>
+          <t>hurt</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -1249,10 +1249,10 @@
     </row>
     <row r="43">
       <c r="B43" t="n">
-        <v>7003</v>
+        <v>3007</v>
       </c>
       <c r="C43" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -1268,14 +1268,14 @@
     </row>
     <row r="44">
       <c r="B44" t="n">
-        <v>7004</v>
+        <v>4000</v>
       </c>
       <c r="C44" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -1287,14 +1287,14 @@
     </row>
     <row r="45">
       <c r="B45" t="n">
-        <v>8000</v>
+        <v>4001</v>
       </c>
       <c r="C45" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>talk</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -1306,14 +1306,14 @@
     </row>
     <row r="46">
       <c r="B46" t="n">
-        <v>9000</v>
+        <v>4002</v>
       </c>
       <c r="C46" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>talk2</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -1325,14 +1325,14 @@
     </row>
     <row r="47">
       <c r="B47" t="n">
-        <v>9001</v>
+        <v>5000</v>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>idle1</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -1344,14 +1344,14 @@
     </row>
     <row r="48">
       <c r="B48" t="n">
-        <v>10000</v>
+        <v>5001</v>
       </c>
       <c r="C48" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>idle1</t>
+          <t>think1</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -1363,14 +1363,14 @@
     </row>
     <row r="49">
       <c r="B49" t="n">
-        <v>10001</v>
+        <v>5002</v>
       </c>
       <c r="C49" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>idle2</t>
+          <t>talk</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -1382,14 +1382,14 @@
     </row>
     <row r="50">
       <c r="B50" t="n">
-        <v>10002</v>
+        <v>5003</v>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>idle3</t>
+          <t>idle1</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -1401,14 +1401,14 @@
     </row>
     <row r="51">
       <c r="B51" t="n">
-        <v>11000</v>
+        <v>6000</v>
       </c>
       <c r="C51" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>idle1</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -1420,14 +1420,14 @@
     </row>
     <row r="52">
       <c r="B52" t="n">
-        <v>11001</v>
+        <v>6001</v>
       </c>
       <c r="C52" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>idle2</t>
+          <t>think1</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -1439,14 +1439,14 @@
     </row>
     <row r="53">
       <c r="B53" t="n">
-        <v>11002</v>
+        <v>6002</v>
       </c>
       <c r="C53" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>idle3</t>
+          <t>talk</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -1458,14 +1458,14 @@
     </row>
     <row r="54">
       <c r="B54" t="n">
-        <v>12000</v>
+        <v>6003</v>
       </c>
       <c r="C54" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>talk2</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -1477,14 +1477,14 @@
     </row>
     <row r="55">
       <c r="B55" t="n">
-        <v>12001</v>
+        <v>6004</v>
       </c>
       <c r="C55" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>idle1</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -1496,10 +1496,10 @@
     </row>
     <row r="56">
       <c r="B56" t="n">
-        <v>2003</v>
+        <v>7000</v>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -1515,18 +1515,18 @@
     </row>
     <row r="57">
       <c r="B57" t="n">
-        <v>2004</v>
+        <v>7001</v>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -1534,18 +1534,18 @@
     </row>
     <row r="58">
       <c r="B58" t="n">
-        <v>2005</v>
+        <v>7002</v>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>attack2</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -1553,10 +1553,10 @@
     </row>
     <row r="59">
       <c r="B59" t="n">
-        <v>2006</v>
+        <v>7003</v>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -1572,18 +1572,18 @@
     </row>
     <row r="60">
       <c r="B60" t="n">
-        <v>3003</v>
+        <v>7004</v>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>idle</t>
+          <t>walk</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -1591,18 +1591,18 @@
     </row>
     <row r="61">
       <c r="B61" t="n">
-        <v>3004</v>
+        <v>8000</v>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>walk</t>
+          <t>idle1</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -1610,18 +1610,18 @@
     </row>
     <row r="62">
       <c r="B62" t="n">
-        <v>3005</v>
+        <v>8001</v>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>idle2</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -1629,18 +1629,18 @@
     </row>
     <row r="63">
       <c r="B63" t="n">
-        <v>3006</v>
+        <v>8002</v>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>hurt</t>
+          <t>idle3</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -1648,20 +1648,210 @@
     </row>
     <row r="64">
       <c r="B64" t="n">
-        <v>3007</v>
+        <v>9000</v>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>die</t>
+          <t>idle</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C65" t="n">
+        <v>9</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>idle1</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C66" t="n">
+        <v>10</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>idle1</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="n">
+        <v>10001</v>
+      </c>
+      <c r="C67" t="n">
+        <v>10</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>idle2</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="n">
+        <v>10002</v>
+      </c>
+      <c r="C68" t="n">
+        <v>10</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>idle3</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C69" t="n">
+        <v>11</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>idle1</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="n">
+        <v>11001</v>
+      </c>
+      <c r="C70" t="n">
+        <v>11</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>idle2</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="n">
+        <v>11002</v>
+      </c>
+      <c r="C71" t="n">
+        <v>11</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>idle3</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C72" t="n">
+        <v>12</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>idle</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="n">
+        <v>12001</v>
+      </c>
+      <c r="C73" t="n">
+        <v>12</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>walk</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="n">
+        <v>13000</v>
+      </c>
+      <c r="C74" t="n">
+        <v>13</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>idle</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>